<commit_message>
Deploying to gh-pages from  @ 156c822df7923b3614dd130c2a7c01efe1b0bfb3 🚀
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/ReportingOrganisation.xlsx
+++ b/api/clv1/codelist/ReportingOrganisation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3835" uniqueCount="2558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3838" uniqueCount="2560">
   <si>
     <t>code</t>
   </si>
@@ -7682,6 +7682,12 @@
   </si>
   <si>
     <t>Forest Trends Association</t>
+  </si>
+  <si>
+    <t>GB-COH-02515034</t>
+  </si>
+  <si>
+    <t>Timber Trade Federation Ltd.</t>
   </si>
   <si>
     <t>US-EIN-13-4052259</t>
@@ -8019,7 +8025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1277"/>
+  <dimension ref="A1:G1278"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -22081,6 +22087,17 @@
         <v>9</v>
       </c>
     </row>
+    <row r="1278" spans="1:4">
+      <c r="A1278" t="s">
+        <v>2558</v>
+      </c>
+      <c r="B1278" t="s">
+        <v>2559</v>
+      </c>
+      <c r="D1278" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploying to gh-pages from  @ 0eb6076fcb156dc6f646c8bb7efd15d31062733d 🚀
</commit_message>
<xml_diff>
--- a/api/clv1/codelist/ReportingOrganisation.xlsx
+++ b/api/clv1/codelist/ReportingOrganisation.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3862" uniqueCount="2575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3865" uniqueCount="2577">
   <si>
     <t>code</t>
   </si>
@@ -7739,6 +7739,12 @@
   </si>
   <si>
     <t>Media Development Investment Fund</t>
+  </si>
+  <si>
+    <t>BE-BCE_KBO-0464147473</t>
+  </si>
+  <si>
+    <t>Laïcité et Humanisme en Afrique Centrale (LHAC)</t>
   </si>
 </sst>
 </file>
@@ -8070,7 +8076,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1286"/>
+  <dimension ref="A1:G1287"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -22231,6 +22237,17 @@
         <v>9</v>
       </c>
     </row>
+    <row r="1287" spans="1:4">
+      <c r="A1287" t="s">
+        <v>2575</v>
+      </c>
+      <c r="B1287" t="s">
+        <v>2576</v>
+      </c>
+      <c r="D1287" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>